<commit_message>
Enhance verification mode analysis
</commit_message>
<xml_diff>
--- a/verification_template.xlsx
+++ b/verification_template.xlsx
@@ -171,6 +171,16 @@
           <t>총액</t>
         </is>
       </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>조건식</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -333,6 +343,16 @@
           <t>75000</t>
         </is>
       </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>기본형</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -493,6 +513,16 @@
       <c r="AF3" t="inlineStr">
         <is>
           <t>총액</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>기본형 또는 정밀형</t>
         </is>
       </c>
     </row>

</xml_diff>